<commit_message>
Preservar y explicitar autoria de Restaurante Noor, incorporar memoria CLAUDE.md y presentacion Kul
- CLAUDE.md: Instrucciones persistentes fijando la autoria exclusiva para Restaurante Noor (Paco Morales y Paola Gualandi)

- index.html y dossiers: Incorporacion de comentarios de cabecera, metadatos y bylines de autoria

- 02_Propuesta_Noor_Kul: Presentacion exportada en HTML/PDF y documento de enlaces

- Actualizacion de indices de articulos y reglas de ignorado
</commit_message>
<xml_diff>
--- a/01_Articulos_PDF/_INDICE_articulos.xlsx
+++ b/01_Articulos_PDF/_INDICE_articulos.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indice" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por carpeta" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Créditos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Indice'!$A$1:$K$42</definedName>
@@ -86,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -100,6 +101,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2456,4 +2460,70 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>¡Come! (كُلْ · Kul) · Cerámica andalusí del siglo XI, epigrafía cúfica y propuesta gastronómica para Restaurante Noor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Autoría</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Autoría: Restaurante Noor · Dirección y supervisión: Paco Morales y Paola Gualandi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Documentos enlazados</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Los PDF de esta carpeta son obras de sus autores y editoriales, que conservan sus derechos. Se han descargado de fuentes de acceso abierto y se usan según sus licencias. La autoría de Noor corresponde a la selección, la organización y este índice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Octubre de 2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>